<commit_message>
cleanup and flexible start stuff
</commit_message>
<xml_diff>
--- a/data/manipulation_tasks_easy.xlsx
+++ b/data/manipulation_tasks_easy.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qtcc\OneDrive\Desktop\rvl\llm_rl_for_manipulation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1FCF91C-A196-49CC-89B5-5D6566AC0777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96030E26-115D-41E1-BD6D-8024AE46542F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="35">
   <si>
     <t>Text Question</t>
   </si>
@@ -57,9 +57,6 @@
     <t>(0.25,0.25,0.02)</t>
   </si>
   <si>
-    <t>category</t>
-  </si>
-  <si>
     <t xml:space="preserve">Take the red block and move it to the position (0,0.375). </t>
   </si>
   <si>
@@ -118,6 +115,21 @@
   </si>
   <si>
     <t>Pick up the block that is the color of a lemon and move it directly between the block with the color of grass and the block with the color of the sky</t>
+  </si>
+  <si>
+    <t>red_cube_start</t>
+  </si>
+  <si>
+    <t>blue_cube_start</t>
+  </si>
+  <si>
+    <t>yellow_cube_start</t>
+  </si>
+  <si>
+    <t>green_cube_start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Take the green block and move it to the position (0,0.375). </t>
   </si>
 </sst>
 </file>
@@ -435,17 +447,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="121.140625" customWidth="1"/>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" customWidth="1"/>
-    <col min="4" max="4" width="21.42578125" customWidth="1"/>
-    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
+    <col min="7" max="7" width="16.140625" customWidth="1"/>
+    <col min="8" max="8" width="17.7109375" customWidth="1"/>
+    <col min="9" max="9" width="17.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -462,12 +478,21 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>11</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -481,13 +506,22 @@
       <c r="E2" t="s">
         <v>8</v>
       </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -501,13 +535,22 @@
       <c r="E3" t="s">
         <v>8</v>
       </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -521,311 +564,485 @@
       <c r="E4" t="s">
         <v>8</v>
       </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>14</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
         <v>5</v>
       </c>
-      <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" t="s">
+        <v>6</v>
+      </c>
+      <c r="H7" t="s">
+        <v>7</v>
+      </c>
+      <c r="I7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>15</v>
       </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" t="s">
+        <v>7</v>
+      </c>
+      <c r="I8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>16</v>
       </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
         <v>17</v>
       </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="D9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H9" t="s">
+        <v>7</v>
+      </c>
+      <c r="I9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="D8" t="s">
-        <v>7</v>
-      </c>
-      <c r="E8" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>19</v>
       </c>
-      <c r="B9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" t="s">
         <v>20</v>
       </c>
-      <c r="B10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>21</v>
       </c>
-      <c r="E10" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H12" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>22</v>
       </c>
-      <c r="B11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" t="s">
-        <v>8</v>
-      </c>
-      <c r="F11">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+      <c r="G13" t="s">
+        <v>6</v>
+      </c>
+      <c r="H13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>23</v>
       </c>
-      <c r="B12" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D14" t="s">
+        <v>20</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G14" t="s">
+        <v>6</v>
+      </c>
+      <c r="H14" t="s">
+        <v>7</v>
+      </c>
+      <c r="I14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>24</v>
       </c>
-      <c r="B13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" t="s">
-        <v>21</v>
-      </c>
-      <c r="E13" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="B15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+      <c r="G15" t="s">
+        <v>6</v>
+      </c>
+      <c r="H15" t="s">
+        <v>7</v>
+      </c>
+      <c r="I15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>25</v>
       </c>
-      <c r="B14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" t="s">
-        <v>8</v>
-      </c>
-      <c r="F14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+      <c r="G16" t="s">
+        <v>6</v>
+      </c>
+      <c r="H16" t="s">
+        <v>7</v>
+      </c>
+      <c r="I16" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>26</v>
       </c>
-      <c r="B15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E15" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+      <c r="G17" t="s">
+        <v>6</v>
+      </c>
+      <c r="H17" t="s">
+        <v>7</v>
+      </c>
+      <c r="I17" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>27</v>
       </c>
-      <c r="B16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16" t="s">
-        <v>8</v>
-      </c>
-      <c r="F16">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+      <c r="G18" t="s">
+        <v>6</v>
+      </c>
+      <c r="H18" t="s">
+        <v>7</v>
+      </c>
+      <c r="I18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>28</v>
       </c>
-      <c r="B17" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" t="s">
-        <v>8</v>
-      </c>
-      <c r="F17">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="B19" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" t="s">
+        <v>6</v>
+      </c>
+      <c r="D19" t="s">
+        <v>7</v>
+      </c>
+      <c r="E19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+      <c r="G19" t="s">
+        <v>6</v>
+      </c>
+      <c r="H19" t="s">
+        <v>7</v>
+      </c>
+      <c r="I19" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>29</v>
       </c>
-      <c r="B18" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" t="s">
-        <v>7</v>
-      </c>
-      <c r="E18" t="s">
-        <v>8</v>
-      </c>
-      <c r="F18">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" t="s">
-        <v>21</v>
-      </c>
-      <c r="E19" t="s">
-        <v>8</v>
-      </c>
-      <c r="F19">
-        <v>6</v>
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" t="s">
+        <v>20</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+      <c r="G20" t="s">
+        <v>6</v>
+      </c>
+      <c r="H20" t="s">
+        <v>7</v>
+      </c>
+      <c r="I20" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>